<commit_message>
Sprint 2 planning: low level design decisions regarding JUMP01
</commit_message>
<xml_diff>
--- a/docs/project-management/Future-scope-lab-enhancements.xlsx
+++ b/docs/project-management/Future-scope-lab-enhancements.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d752cb73b61fc091/Desktop/linuxlabs/projectredstone/docs/project-management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{BE0CC9B9-D038-4FB1-8848-D1A2A3D5E109}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D52D4EB-4DD9-4FB4-A27B-B6D9A507F701}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{BE0CC9B9-D038-4FB1-8848-D1A2A3D5E109}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E0AE4AC-6BFE-43D4-9493-9ADDC5B568B2}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{62DA3A3F-4F63-419A-9568-3A15DBCDC23A}"/>
+    <workbookView xWindow="2640" yWindow="2640" windowWidth="21600" windowHeight="11295" xr2:uid="{62DA3A3F-4F63-419A-9568-3A15DBCDC23A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="278">
   <si>
     <t>Ref</t>
   </si>
@@ -867,6 +867,12 @@
   </si>
   <si>
     <t>FC-049</t>
+  </si>
+  <si>
+    <t>Future consideration — Dedicated Hypervisor Management Network</t>
+  </si>
+  <si>
+    <t>FC-050</t>
   </si>
 </sst>
 </file>
@@ -942,6 +948,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1261,7 +1271,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F606E89-1784-4BEF-8D33-90F342977587}">
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr defaultColWidth="109.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.140625" bestFit="1" customWidth="1"/>
@@ -2260,6 +2270,14 @@
         <v>274</v>
       </c>
     </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="B51" t="s">
+        <v>276</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>